<commit_message>
feat(pangea): gambar materi dibuat PENUH memenuhi ruang + daftar soal dibuat ulang
Permintaan pemilik proyek:
1. 'yang di ss an kedua kamu bikin full deh gambarnya' - gambar Pangea dari dosen
   (public/images.jpg) sebelumnya tampil kecil di tengah karena memakai
   object-contain, padahal gambarnya tegak (960x1280) sedangkan ruangnya mendatar.
   Sekarang memakai w-full h-full object-cover sehingga memenuhi seluruh ruang.
2. 'bikinin list soal dan jawaban yang sekarang, baik di level 1 dan 2' - daftar
   soal dibuat ULANG dari bank yang sekarang: 107 baris Wordle dan 72 baris TTS.
   Daftar sebelumnya sempat BASI karena dibuat sebelum jawaban dikembalikan ke set
   asli; itu salah saya karena tidak memperkirakannya.

Diverifikasi: berkas xlsx memuat jawaban set ASLI (LITOSFER, ASTENOSFER, GEODYNAMO,
SEISMOGRAF, SANANDREAS, INTIDALAM, AMBULANS, MENDATAR) dan tidak lagi memuat jawaban
hasil penyelarasan (SIAL, SIMA, PEMATANG, GOGGLE, PRESENSI, HUNIAN, KORSLETING).
</commit_message>
<xml_diff>
--- a/Daftar-Soal-RESQ-BOX.xlsx
+++ b/Daftar-Soal-RESQ-BOX.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -501,12 +501,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lapisan paling luar bumi tempat kita tinggal, dan paling tipis.</t>
+          <t>Lapisan paling luar bumi tempat kita tinggal, dan merupakan lapisan yang paling tipis.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Bagian terluar bumi yang menjadi tempat berpijak seluruh makhluk hidup.</t>
+          <t>Bagian terluar bumi yang paling tipis, tempat kita berpijak.</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Jenis kerak bumi di bawah daratan, tebalnya sampai 100 kilometer.</t>
+          <t>Jenis kerak bumi di bawah daratan yang memiliki ketebalan mencapai 100 kilometer.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Kerak di bawah daratan; paling tebal di antara kedua jenis kerak.</t>
+          <t>Daratan yang sangat luas; kerak bumi di bawahnya paling tebal, sampai 100 km.</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Kerak di bawah lautan; hanya 5-15 km tetapi paling berat.</t>
+          <t>Lautan yang sangat luas; kerak di bawahnya hanya 5-15 km tetapi lebih berat.</t>
         </is>
       </c>
     </row>
@@ -580,17 +580,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GRANIT</t>
+          <t>LITOSFER</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Batuan penyusun kerak benua, berwarna terang dan lebih ringan.</t>
+          <t>Lapisan batuan paling luar bumi, tersusun dari kerak dan bagian atas mantel.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Batuan pembentuk kerak di bawah daratan, bersifat ringan.</t>
+          <t>Lapisan kaku terluar bumi, gabungan kerak dengan bagian atas mantel.</t>
         </is>
       </c>
     </row>
@@ -608,17 +608,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BASAL</t>
+          <t>DARATAN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Batuan penyusun kerak samudra, berwarna gelap dan lebih padat.</t>
+          <t>Wilayah kerak bumi yang letaknya lebih tinggi daripada permukaan laut.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Batuan pembentuk kerak di bawah lautan, bersifat padat dan berat.</t>
+          <t>Bagian permukaan bumi yang kering dan tidak tertutup air.</t>
         </is>
       </c>
     </row>
@@ -636,17 +636,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TIPIS</t>
+          <t>LAUTAN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Kerak samudra bersifat ... dibandingkan kerak benua.</t>
+          <t>Wilayah kerak bumi yang tertutup air, keraknya lebih tipis tetapi lebih berat.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Sifat kerak di bawah lautan: hanya 5-15 kilometer tebalnya.</t>
+          <t>Bagian bumi yang tergenang air asin dan menutupi sebagian besar permukaannya.</t>
         </is>
       </c>
     </row>
@@ -664,17 +664,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TEBAL</t>
+          <t>TIPIS</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Kerak benua bersifat ... dibandingkan kerak samudra.</t>
+          <t>Kerak samudra bersifat ... dibandingkan kerak benua.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sifat kerak di bawah daratan: mencapai 30-100 kilometer.</t>
+          <t>Sifat kerak di bawah lautan jika dibandingkan kerak di bawah daratan.</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>PADAT</t>
+          <t>GRANIT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sifat lapisan kerak bumi yang tersusun dari batuan.</t>
+          <t>Batuan penyusun utama kerak benua, berwarna lebih terang dan lebih ringan.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sifat lapisan terluar bumi karena terbuat dari batuan, bukan zat alir.</t>
+          <t>Jenis batuan yang mendominasi kerak di bawah daratan; warnanya terang.</t>
         </is>
       </c>
     </row>
@@ -720,17 +720,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>BERAT</t>
+          <t>BASAL</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sifat kerak samudra selain lebih padat, dibandingkan kerak benua.</t>
+          <t>Batuan penyusun utama kerak samudra, berwarna gelap dan lebih padat.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sifat kerak di bawah lautan yang membuatnya tenggelam lebih dalam.</t>
+          <t>Jenis batuan yang mendominasi kerak di bawah lautan; warnanya gelap.</t>
         </is>
       </c>
     </row>
@@ -748,17 +748,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LAPISAN</t>
+          <t>INDONESIA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Kerak bumi disebut sebagai ... paling luar dari bumi.</t>
+          <t>Negara yang terletak di pertemuan Lempeng Indo-Australia, Eurasia, dan Pasifik.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sebutan bagi kerak: bagian teratas yang menyusun tubuh bumi.</t>
+          <t>Negara kita, berada di titik pertemuan tiga lempeng besar sehingga rawan gempa.</t>
         </is>
       </c>
     </row>
@@ -776,17 +776,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>SUHU</t>
+          <t>SUMATRA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Besaran yang berkisar 25 sampai 500 derajat Celsius di kerak bumi.</t>
+          <t>Pulau yang tanahnya subur karena abu vulkanik, tetapi juga rawan gempa.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Besaran yang diukur termometer; di kerak bumi nilainya 25-500 derajat.</t>
+          <t>Pulau di barat negara kita; tanahnya subur, tetapi sering diguncang gempa.</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>LUAR</t>
+          <t>GEMPA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Kedudukan kerak bumi: lapisan paling ... dari bumi.</t>
+          <t>Peristiwa yang sering terjadi di Indonesia karena lempengnya saling bertumbukan.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Kedudukan kerak dibandingkan seluruh lapisan bumi lainnya.</t>
+          <t>Getaran yang menjalar di permukaan bumi akibat lempeng yang bertumbukan.</t>
         </is>
       </c>
     </row>
@@ -832,17 +832,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>RINGAN</t>
+          <t>TEBAL</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sifat batuan granit penyusun kerak benua, selain berwarna terang.</t>
+          <t>Kerak benua bersifat ... dibandingkan kerak samudra.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Sifat granit yang membuat kerak benua mengapung di atas kerak samudra.</t>
+          <t>Sifat kerak di bawah daratan jika dibandingkan kerak di bawah lautan.</t>
         </is>
       </c>
     </row>
@@ -860,17 +860,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SIAL</t>
+          <t>SEDIMEN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Nama lain kerak benua berdasarkan unsur penyusunnya: silika dan aluminium.</t>
+          <t>Batuan yang terbentuk dari endapan material di permukaan kerak.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Sebutan kerak benua dari dua unsur pembentuknya, silika dan aluminium.</t>
+          <t>Endapan yang mengeras lapis demi lapis di permukaan bumi.</t>
         </is>
       </c>
     </row>
@@ -888,185 +888,185 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SIMA</t>
+          <t>LEMPENG</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Nama lain kerak samudra berdasarkan unsur penyusunnya: silika dan magnesium.</t>
+          <t>Pecahan besar kerak bumi yang bergerak di atas lapisan yang kental.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Sebutan kerak samudra dari dua unsur pembentuknya, silika dan magnesium.</t>
+          <t>Potongan raksasa kerak bumi yang saling bergerak dan bertumbukan.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mantel Bumi</t>
+          <t>Kerak Bumi</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MANTEL</t>
+          <t>KERAS</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Lapisan di bawah kerak bumi yang merupakan lapisan paling tebal (2.900 km).</t>
+          <t>Sifat lapisan paling luar bumi yang membuat kita dapat berpijak di atasnya.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Lapisan tertebal di dalam bumi, letaknya tepat di bawah kerak.</t>
+          <t>Sifat batuan di permukaan sehingga kita dapat berdiri di atasnya.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mantel Bumi</t>
+          <t>Kerak Bumi</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KONVEKSI</t>
+          <t>SILIKAT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Arus perputaran panas di dalam mantel yang menggerakkan lempeng bumi.</t>
+          <t>Senyawa pembentuk batuan yang banyak menyusun lapisan padat bumi.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Perpindahan panas yang berputar membentuk sel, dan menjadi tenaga penggerak lempeng.</t>
+          <t>Senyawa batuan yang mengandung silikon dan oksigen, banyak menyusun bumi.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mantel Bumi</t>
+          <t>Kerak Bumi</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ADONAN</t>
+          <t>BATU</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Material mantel paling mirip benda kental ini, sehingga dapat mengalir sangat lambat.</t>
+          <t>Benda padat alami yang menyusun lapisan kerak bumi.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Material mantel diibaratkan seperti campuran tepung dan air yang kental ini.</t>
+          <t>Bahan padat alami pembentuk kerak, misalnya granit dan basal.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mantel Bumi</t>
+          <t>Kerak Bumi</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>FLUIDA</t>
+          <t>LERENG</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Wujud material mantel: bukan padat kaku, melainkan ... sangat kental.</t>
+          <t>Sisi miring sebuah gunung atau bukit, dari kaki sampai ke puncaknya.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Sebutan untuk zat yang dapat mengalir, misalnya zat kental di dalam mantel.</t>
+          <t>Bagian miring gunung yang menghubungkan kaki dengan puncaknya.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mantel Bumi</t>
+          <t>Kerak Bumi</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ARUS</t>
+          <t>TANAH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Aliran panas yang terbentuk di dalam mantel karena pemanasan dari bawah.</t>
+          <t>Lapisan paling atas kerak bumi tempat tumbuhan tumbuh dan berakar.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Yang mengalir dan berputar di dalam mantel, menjadi tenaga penggerak lempeng.</t>
+          <t>Lapisan gembur di permukaan tempat akar tumbuhan menancap.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mantel Bumi</t>
+          <t>Kerak Bumi</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PANAS</t>
+          <t>LEMPUNG</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Suhu mantel berkisar 1.000 sampai 3.700 derajat Celsius, artinya mantel sangat...</t>
+          <t>Jenis tanah yang lengket dan kedap air, sering dipakai membuat kerajinan.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Keadaan suhu di dalam mantel yang mencapai ribuan derajat Celsius.</t>
+          <t>Jenis tanah yang liat dan sulit dilalui air; bahan dasar gerabah.</t>
         </is>
       </c>
     </row>
@@ -1080,21 +1080,21 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>KENTAL</t>
+          <t>MANTEL</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sifat material mantel: sangat ... sehingga mengalir sangat lambat.</t>
+          <t>Lapisan di bawah kerak bumi yang merupakan lapisan paling tebal (2.900 km).</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sifat zat yang mengalir lambat karena partikelnya rapat, seperti material mantel.</t>
+          <t>Lapisan tertebal di dalam bumi, letaknya tepat di bawah kerak.</t>
         </is>
       </c>
     </row>
@@ -1108,21 +1108,21 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>BERPUTAR</t>
+          <t>KONVEKSI</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Gerakan aliran panas mantel yang berbalik arah membentuk lingkaran.</t>
+          <t>Arus perputaran panas di dalam mantel yang menggerakkan lempeng bumi.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sifat gerak aliran panas mantel: naik lalu turun kembali membentuk lingkaran.</t>
+          <t>Perpindahan panas yang berputar membentuk sel, dan menjadi tenaga penggerak lempeng.</t>
         </is>
       </c>
     </row>
@@ -1136,21 +1136,21 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MENDIDIH</t>
+          <t>ADONAN</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Keadaan air di dalam panci saat dipanaskan, dipakai sebagai perumpamaan arus mantel.</t>
+          <t>Material mantel paling mirip benda kental ini, sehingga dapat mengalir sangat lambat.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Perumpamaan arus mantel: seperti air panas yang menggelegak di panci.</t>
+          <t>Material mantel diibaratkan seperti campuran tepung dan air yang kental ini.</t>
         </is>
       </c>
     </row>
@@ -1164,21 +1164,21 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PANCI</t>
+          <t>FLUIDA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Wadah tempat air direbus, dipakai sebagai perumpamaan arus konveksi mantel.</t>
+          <t>Wujud material mantel: bukan padat kaku, melainkan ... sangat kental.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Perkakas dapur untuk merebus air, menjadi perumpamaan sel konveksi.</t>
+          <t>Sebutan untuk zat yang dapat mengalir, misalnya zat kental di dalam mantel.</t>
         </is>
       </c>
     </row>
@@ -1192,21 +1192,21 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>LEMPENG</t>
+          <t>SILIKAT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Bagian kerak bumi yang digerakkan oleh arus panas di dalam mantel.</t>
+          <t>Bahan batuan penyusun mantel bumi.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Kepingan kerak bumi; arus mantel menjadi mesin penggeraknya.</t>
+          <t>Senyawa yang banyak menyusun batuan mantel, mengandung silikon dan oksigen.</t>
         </is>
       </c>
     </row>
@@ -1220,189 +1220,189 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>PENGGERAK</t>
+          <t>PANAS</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Peran arus konveksi mantel bagi pergerakan lempeng bumi: sebagai mesin ...</t>
+          <t>Suhu mantel berkisar 1.000 sampai 3.700 derajat Celsius, artinya mantel sangat...</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Peran arus mantel: menjadi mesin yang menggerakkan lempeng bumi.</t>
+          <t>Keadaan suhu di dalam mantel yang mencapai ribuan derajat Celsius.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Inti Luar</t>
+          <t>Mantel Bumi</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NIKEL</t>
+          <t>KENTAL</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bahan yang menjadi penyusun utama lapisan inti bumi adalah besi dan...</t>
+          <t>Sifat material mantel: sangat ... sehingga mengalir sangat lambat.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Logam berwarna keperakan yang mendampingi besi di pusat bumi.</t>
+          <t>Sifat zat yang mengalir lambat karena partikelnya rapat, seperti material mantel.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Inti Luar</t>
+          <t>Mantel Bumi</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CAIRAN</t>
+          <t>ASTENOSFER</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Inti luar bumi wujudnya berupa...</t>
+          <t>Lapisan kental di bagian atas mantel, tepat di bawah kerak bumi.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Wujud zat yang dapat mengalir, seperti logam panas di inti luar.</t>
+          <t>Bagian paling atas mantel yang paling liat, tempat lempeng bergerak di atasnya.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Inti Luar</t>
+          <t>Mantel Bumi</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MAGNET</t>
+          <t>MELELEH</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Lapisan inti bumi luar menghasilkan medan... yang melindungi bumi dari radiasi matahari.</t>
+          <t>Yang terjadi pada batuan bila suhunya melampaui titik leburnya.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sifat gaya tarik yang dimiliki bumi dan dapat menarik besi.</t>
+          <t>Perubahan wujud batuan menjadi zat alir karena suhunya sangat tinggi.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Inti Luar</t>
+          <t>Mantel Bumi</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>BESI</t>
+          <t>SIRKULASI</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Logam utama penyusun inti bumi, bersama nikel.</t>
+          <t>Nama lain perputaran aliran panas yang membentuk sel di dalam mantel.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Logam yang paling banyak menyusun pusat bumi, bersama nikel.</t>
+          <t>Gerakan berputar aliran zat kental di dalam mantel, dari bawah ke atas lalu kembali turun.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Inti Luar</t>
+          <t>Mantel Bumi</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>PUTARAN</t>
+          <t>KONDUKSI</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Gerakan berulang aliran logam cair di inti luar yang membangkitkan magnet.</t>
+          <t>Perpindahan panas melalui sebuah zat tanpa memindahkan zatnya sendiri.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Gerak berulang logam cair inti luar; inilah yang menimbulkan medan magnet.</t>
+          <t>Cara panas merambat melalui sebuah benda tanpa benda itu ikut berpindah.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Inti Luar</t>
+          <t>Mantel Bumi</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EKSTREM</t>
+          <t>GEOTERMAL</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Sifat panas di inti luar yang membuat logam besi dan nikel meleleh.</t>
+          <t>Sebutan bagi energi panas yang berasal dari dalam bumi.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sifat suhu inti luar yang melampaui titik leleh besi dan nikel.</t>
+          <t>Istilah bagi panas bumi yang dimanfaatkan sebagai pembangkit listrik.</t>
         </is>
       </c>
     </row>
@@ -1416,21 +1416,21 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LOGAM</t>
+          <t>NIKEL</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Inti bumi tersusun dari ... besi dan nikel, bukan batuan.</t>
+          <t>Bahan yang menjadi penyusun utama lapisan inti bumi adalah besi dan...</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Bahan penghantar panas dan listrik yang baik, seperti besi dan nikel.</t>
+          <t>Logam berwarna keperakan yang mendampingi besi di pusat bumi.</t>
         </is>
       </c>
     </row>
@@ -1444,21 +1444,21 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>PANAS</t>
+          <t>CAIRAN</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Suhu inti luar sekitar 5.000 derajat Celsius, artinya sangat...</t>
+          <t>Inti luar bumi wujudnya berupa...</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Keadaan suhu di inti luar yang mencapai sekitar 5.000 derajat Celsius.</t>
+          <t>Wujud zat yang dapat mengalir, seperti logam panas di inti luar.</t>
         </is>
       </c>
     </row>
@@ -1472,21 +1472,21 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>DINAMO</t>
+          <t>MAGNET</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Alat pembangkit listrik; perputaran logam inti luar bekerja seperti ini.</t>
+          <t>Lapisan inti bumi luar menghasilkan medan... yang melindungi bumi dari radiasi matahari.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Perumpamaan bagi kerja inti luar: seperti ... raksasa yang berputar.</t>
+          <t>Sifat gaya tarik yang dimiliki bumi dan dapat menarik besi.</t>
         </is>
       </c>
     </row>
@@ -1500,21 +1500,21 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>RAKSASA</t>
+          <t>BESI</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Ukuran dinamo yang menggambarkan besarnya medan magnet bumi.</t>
+          <t>Logam utama penyusun inti bumi, bersama nikel.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sifat dinamo yang dibentuk oleh inti luar bumi: sangat besar.</t>
+          <t>Logam yang paling banyak menyusun pusat bumi, bersama nikel.</t>
         </is>
       </c>
     </row>
@@ -1528,21 +1528,21 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>MATAHARI</t>
+          <t>LELEHAN</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Bintang yang radiasinya dibelokkan oleh medan magnet bumi.</t>
+          <t>Inti luar berupa ... logam, karena suhunya melampaui titik leleh besi.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sumber badai radiasi yang ditahan oleh medan magnet bumi.</t>
+          <t>Logam yang telah berubah menjadi zat alir karena panas.</t>
         </is>
       </c>
     </row>
@@ -1556,21 +1556,21 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>LINDUNG</t>
+          <t>KOMPAS</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Medan magnet bumi bertugas ... permukaan dari radiasi angkasa.</t>
+          <t>Alat penunjuk arah yang bekerja karena memanfaatkan medan magnet bumi.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Tugas medan magnet bumi: menahan radiasi angkasa agar tidak sampai ke permukaan.</t>
+          <t>Alat navigasi berjarum yang selalu menunjuk ke arah utara dan selatan.</t>
         </is>
       </c>
     </row>
@@ -1584,21 +1584,21 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>MEDAN</t>
+          <t>LOGAM</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Wilayah yang dipengaruhi sebuah gaya, misalnya gaya magnet bumi.</t>
+          <t>Inti bumi tersusun dari ... besi dan nikel, bukan batuan.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Ruang di sekitar magnet yang masih terpengaruh gaya tariknya.</t>
+          <t>Bahan penghantar panas dan listrik yang baik, seperti besi dan nikel.</t>
         </is>
       </c>
     </row>
@@ -1612,21 +1612,21 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>BADAI</t>
+          <t>PANAS</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Sebutan bagi gangguan radiasi hebat yang datang dari matahari.</t>
+          <t>Suhu inti luar sekitar 5.000 derajat Celsius, artinya sangat...</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Gangguan radiasi matahari yang dibelokkan medan magnet bumi.</t>
+          <t>Keadaan suhu di inti luar yang mencapai sekitar 5.000 derajat Celsius.</t>
         </is>
       </c>
     </row>
@@ -1640,21 +1640,21 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>PERISAI</t>
+          <t>KUTUB</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Sebutan bagi medan magnet bumi karena melindungi dari radiasi angkasa.</t>
+          <t>Medan magnet bumi memiliki dua ..., yaitu utara dan selatan.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Sebutan bagi pelindung alami bumi dari radiasi angkasa.</t>
+          <t>Sebutan bagi ujung utara dan ujung selatan sebuah magnet.</t>
         </is>
       </c>
     </row>
@@ -1668,21 +1668,21 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>RADIASI</t>
+          <t>ARUS</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pancaran berbahaya dari angkasa yang dilindungi medan magnet bumi.</t>
+          <t>Logam cair di inti luar membentuk ... listrik yang menghasilkan medan magnet.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Pancaran berbahaya matahari yang dibelokkan oleh medan magnet bumi.</t>
+          <t>Aliran listrik yang timbul dari logam yang bergerak di inti luar.</t>
         </is>
       </c>
     </row>
@@ -1696,21 +1696,21 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>CAIR</t>
+          <t>LISTRIK</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Wujud logam di inti luar, berbeda dengan inti dalam yang padat.</t>
+          <t>Jenis aliran yang timbul dari logam cair yang bergerak di inti luar.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Wujud zat yang mengalir dan tidak mempertahankan bentuknya.</t>
+          <t>Aliran energi yang muncul dari logam yang bergerak, dan membangkitkan magnet.</t>
         </is>
       </c>
     </row>
@@ -1724,189 +1724,189 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>SUHU</t>
+          <t>LINDUNG</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Besaran yang mencapai 5.000 derajat Celsius di inti luar bumi.</t>
+          <t>Medan magnet bumi bertugas ... permukaan dari radiasi angkasa.</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Besaran yang diukur dengan termometer dan menyatakan derajat panas.</t>
+          <t>Tugas medan magnet bumi: menahan radiasi angkasa agar tidak sampai ke permukaan.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Inti Dalam</t>
+          <t>Inti Luar</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>KRISTAL</t>
+          <t>MEDAN</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Bentuk susunan logam besi dan nikel di inti dalam.</t>
+          <t>Wilayah yang dipengaruhi sebuah gaya, misalnya gaya magnet bumi.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Susunan atom logam yang teratur rapat di inti dalam.</t>
+          <t>Ruang di sekitar magnet yang masih terpengaruh gaya tariknya.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Inti Dalam</t>
+          <t>Inti Luar</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PADAT</t>
+          <t>GEODYNAMO</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Inti dalam berbentuk sangat ... karena tekanan yang sangat besar dari segala arah.</t>
+          <t>Mekanisme perputaran logam di inti luar yang membangkitkan magnet bumi.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Sifat zat yang partikelnya rapat dan tidak dapat mengalir, seperti lapisan terdalam bumi.</t>
+          <t>Cara kerja perputaran logam panas di inti luar sehingga bumi memiliki magnet.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Inti Dalam</t>
+          <t>Inti Luar</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>BESI</t>
+          <t>PERISAI</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Logam utama penyusun bola inti dalam bumi.</t>
+          <t>Sebutan bagi medan magnet bumi karena melindungi dari radiasi angkasa.</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Logam utama pada bola terdalam bumi, berpasangan dengan nikel.</t>
+          <t>Sebutan bagi pelindung alami bumi dari radiasi angkasa.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Inti Dalam</t>
+          <t>Inti Luar</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>TEKANAN</t>
+          <t>LEBUR</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Penyebab inti dalam tetap padat walaupun suhunya 6.000 derajat Celsius.</t>
+          <t>Hancur menjadi zat alir karena panas yang sangat tinggi.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Gaya desak dari segala arah yang membuat bagian terdalam bumi tetap padat.</t>
+          <t>Peristiwa berubahnya logam menjadi zat alir akibat panas yang sangat tinggi.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Inti Dalam</t>
+          <t>Inti Luar</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>BOLA</t>
+          <t>CAIR</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bentuk inti dalam bumi, terselubung oleh inti luar.</t>
+          <t>Wujud logam di inti luar, berbeda dengan inti dalam yang padat.</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Bentuk bulat sempurna seperti yang dimiliki lapisan terdalam bumi.</t>
+          <t>Wujud zat yang mengalir dan tidak mempertahankan bentuknya.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Inti Dalam</t>
+          <t>Inti Luar</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>PUSAT</t>
+          <t>SUHU</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Letak inti dalam: di ... bumi.</t>
+          <t>Besaran yang mencapai 5.000 derajat Celsius di inti luar bumi.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Tempat kedudukan bagian terdalam bumi: di bagian paling tengah.</t>
+          <t>Besaran yang diukur dengan termometer dan menyatakan derajat panas.</t>
         </is>
       </c>
     </row>
@@ -1920,21 +1920,21 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>GRAVITASI</t>
+          <t>INTIDALAM</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Gaya yang menarik segala sesuatu menuju pusat bumi.</t>
+          <t>Lapisan terdalam planet bumi pada kedalaman 6.371 kilometer.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Gaya tarik bumi yang membuat benda jatuh ke bawah.</t>
+          <t>Bagian paling tengah bumi, berupa bola logam di kedalaman 6.371 km.</t>
         </is>
       </c>
     </row>
@@ -1948,21 +1948,21 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ATOM</t>
+          <t>PADAT</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Bagian terkecil penyusun besi yang dikunci rapat oleh tekanan di inti dalam.</t>
+          <t>Inti dalam berbentuk sangat ... karena tekanan yang sangat besar dari segala arah.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Bagian terkecil penyusun logam; di inti dalam terkuci rapat oleh tekanan.</t>
+          <t>Sifat zat yang partikelnya rapat dan tidak dapat mengalir, seperti lapisan terdalam bumi.</t>
         </is>
       </c>
     </row>
@@ -1976,21 +1976,21 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>INTI</t>
+          <t>BESI</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Bagian paling tengah dari sesuatu, misalnya bagian terdalam bumi.</t>
+          <t>Logam utama penyusun bola inti dalam bumi.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Bagian paling tengah, misalnya pada buah atau pada bumi.</t>
+          <t>Logam utama pada bola terdalam bumi, berpasangan dengan nikel.</t>
         </is>
       </c>
     </row>
@@ -2004,21 +2004,21 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>NOL</t>
+          <t>TEKANAN</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Nilai gravitasi tepat di pusat bumi, karena tarikan dari segala arah saling meniadakan.</t>
+          <t>Penyebab inti dalam tetap padat walaupun suhunya 6.000 derajat Celsius.</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Nilai gaya tarik di titik pusat bumi: karena saling meniadakan.</t>
+          <t>Gaya desak dari segala arah yang membuat bagian terdalam bumi tetap padat.</t>
         </is>
       </c>
     </row>
@@ -2032,21 +2032,21 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>NIKEL</t>
+          <t>BOLA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Logam penyusun inti bumi yang berpasangan dengan besi.</t>
+          <t>Bentuk inti dalam bumi, terselubung oleh inti luar.</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Logam berwarna keperakan yang menyertai besi di pusat bumi.</t>
+          <t>Bentuk bulat sempurna seperti yang dimiliki lapisan terdalam bumi.</t>
         </is>
       </c>
     </row>
@@ -2060,189 +2060,189 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>DAHSYAT</t>
+          <t>PUSAT</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Sifat tekanan di inti dalam yang membuat besi tetap padat.</t>
+          <t>Letak inti dalam: di ... bumi.</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Sifat tekanan dari seluruh bumi yang mengunci besi tetap padat.</t>
+          <t>Tempat kedudukan bagian terdalam bumi: di bagian paling tengah.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Batas Divergen</t>
+          <t>Inti Dalam</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>PANGEA</t>
+          <t>GRAVITASI</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Nama superbenua raksasa purba yang dulunya menyatukan seluruh daratan bumi.</t>
+          <t>Gaya yang menarik segala sesuatu menuju pusat bumi.</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Benua raksasa purba yang dahulu menyatukan seluruh daratan dunia.</t>
+          <t>Gaya tarik bumi yang membuat benda jatuh ke bawah.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Batas Divergen</t>
+          <t>Inti Dalam</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>MENJAUH</t>
+          <t>TERDALAM</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Arah pergerakan dua lempeng tektonik pada batas divergen saling...</t>
+          <t>Inti dalam adalah lapisan yang paling ... di seluruh bumi.</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Arah gerak dua lempeng pada batas divergen, yaitu saling meninggalkan.</t>
+          <t>Kedudukan lapisan yang paling jauh dari permukaan bumi.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Inti Dalam</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
         <v>5</v>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Batas Divergen</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>1</v>
-      </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>MAGMA</t>
+          <t>INTI</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Batuan cair panas dari mantel bumi yang menerobos naik mengisi celah rekahan lempeng.</t>
+          <t>Bagian paling tengah dari sesuatu, misalnya bagian terdalam bumi.</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Zat cair panas dari dalam bumi yang naik mengisi rekahan kerak.</t>
+          <t>Bagian paling tengah, misalnya pada buah atau pada bumi.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
+        <v>4</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Inti Dalam</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
         <v>5</v>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Batas Divergen</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>2</v>
-      </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>DIVERGEN</t>
+          <t>PADUAN</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Nama batas lempeng tempat dua lempeng bergerak saling menjauh.</t>
+          <t>Campuran dua logam atau lebih, seperti besi dan nikel di pusat bumi.</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Sebutan batas lempeng yang kedua sisinya bergerak saling meninggalkan.</t>
+          <t>Hasil pencampuran beberapa logam, misalnya besi dengan nikel.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Batas Divergen</t>
+          <t>Inti Dalam</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>HANYUT</t>
+          <t>NIKEL</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Peristiwa terpisahnya benua setelah Pangea retak, menurut teori Alfred Wegener.</t>
+          <t>Logam penyusun inti bumi yang berpasangan dengan besi.</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Yang dialami benua setelah Pangea retak dan bergerak saling menjauh.</t>
+          <t>Logam berwarna keperakan yang menyertai besi di pusat bumi.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Batas Divergen</t>
+          <t>Inti Dalam</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>LEMPENG</t>
+          <t>MAMPAT</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Kepingan kerak bumi yang terus bergerak perlahan di atas mantel.</t>
+          <t>Keadaan zat yang partikelnya sangat rapat karena tekanan yang besar.</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Bagian kerak bumi yang terpecah dan bergerak perlahan di atas mantel.</t>
+          <t>Keadaan zat yang partikelnya terdesak sangat rapat oleh tekanan besar.</t>
         </is>
       </c>
     </row>
@@ -2256,21 +2256,21 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>TEKTONIK</t>
+          <t>PANGEA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Sebutan bagi lempeng yang bergerak perlahan di atas mantel bumi.</t>
+          <t>Nama superbenua raksasa purba yang dulunya menyatukan seluruh daratan bumi.</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Jenis lempeng yang bergerak perlahan di atas mantel, penggerak benua.</t>
+          <t>Benua raksasa purba yang dahulu menyatukan seluruh daratan dunia.</t>
         </is>
       </c>
     </row>
@@ -2284,21 +2284,21 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>MENDESAK</t>
+          <t>MENJAUH</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Yang dilakukan magma panas terhadap permukaan bumi saat naik.</t>
+          <t>Arah pergerakan dua lempeng tektonik pada batas divergen saling...</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Perbuatan magma panas yang naik lalu menekan permukaan bumi.</t>
+          <t>Arah gerak dua lempeng pada batas divergen, yaitu saling meninggalkan.</t>
         </is>
       </c>
     </row>
@@ -2312,21 +2312,21 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>SAMUDRA</t>
+          <t>MAGMA</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Batas divergen paling banyak terdapat di dasar...</t>
+          <t>Batuan cair panas dari mantel bumi yang menerobos naik mengisi celah rekahan lempeng.</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Batas divergen paling banyak ditemukan di dasar lautan luas.</t>
+          <t>Zat cair panas dari dalam bumi yang naik mengisi rekahan kerak.</t>
         </is>
       </c>
     </row>
@@ -2340,21 +2340,21 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>MENDINGIN</t>
+          <t>DIVERGEN</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Yang terjadi pada magma setelah keluar ke permukaan bumi.</t>
+          <t>Nama batas lempeng tempat dua lempeng bergerak saling menjauh.</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Proses yang dialami magma setelah naik, sebelum mengeras menjadi batuan.</t>
+          <t>Sebutan batas lempeng yang kedua sisinya bergerak saling meninggalkan.</t>
         </is>
       </c>
     </row>
@@ -2368,21 +2368,21 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>TENGAH</t>
+          <t>CELAH</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Batas divergen di dasar samudra disebut punggung ... samudra.</t>
+          <t>Ruang terbuka yang terbentuk saat dua lempeng saling menjauh, lalu terisi magma.</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Batas divergen di dasar laut disebut punggung ... laut.</t>
+          <t>Rongga terbuka di kerak yang muncul ketika lempeng saling bergerak menjauh.</t>
         </is>
       </c>
     </row>
@@ -2396,21 +2396,21 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>MENGERAS</t>
+          <t>REKAHAN</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Yang terjadi pada magma setelah mendingin di permukaan.</t>
+          <t>Retakan pada kerak bumi tempat magma dapat naik ke permukaan.</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Perubahan magma setelah dingin, menjadi batuan kerak baru.</t>
+          <t>Belahan pada kerak bumi yang menjadi jalan naiknya zat cair panas.</t>
         </is>
       </c>
     </row>
@@ -2424,21 +2424,21 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>PEMATANG</t>
+          <t>MEMISAH</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Bentuk dasar laut yang menjulang di tengah samudra akibat batas divergen.</t>
+          <t>Arti kata divergen: kedua lempeng saling...</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Bentuk dasar laut yang naik di tengah samudra, disebut mid-ocean ridge.</t>
+          <t>Arti kata divergen: kedua lempeng saling meninggalkan satu sama lain.</t>
         </is>
       </c>
     </row>
@@ -2452,21 +2452,21 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>RETAK</t>
+          <t>PUNGGUNG</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Keadaan kerak yang terbelah akibat gaya yang menariknya memisah.</t>
+          <t>Bentuk dasar samudra yang menjulang di batas divergen: ... tengah samudra.</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Keadaan kerak yang terbelah-belah karena ditarik ke dua arah.</t>
+          <t>Bagian dasar laut yang meninggi di batas divergen, disebut ... tengah samudra.</t>
         </is>
       </c>
     </row>
@@ -2480,21 +2480,21 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>MEMPERLUAS</t>
+          <t>SAMUDRA</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Yang dilakukan dasar laut ketika magma baru terus menambah kerak.</t>
+          <t>Batas divergen paling banyak terdapat di dasar...</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Akibat magma baru yang terus keluar: dasar laut bertambah lebar.</t>
+          <t>Batas divergen paling banyak ditemukan di dasar lautan luas.</t>
         </is>
       </c>
     </row>
@@ -2508,21 +2508,21 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>PERLAHAN</t>
+          <t>TERBELAH</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Sifat gerak lempeng tektonik menurut teori Alfred Wegener.</t>
+          <t>Daratan Pangea perlahan ... menjadi benua-benua yang kita kenal sekarang.</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Cara lempeng tektonik bergerak: sangat lambat sehingga tidak terasa.</t>
+          <t>Benua yang kita kenal sekarang dahulu menyatu, lalu saling melepaskan diri.</t>
         </is>
       </c>
     </row>
@@ -2536,21 +2536,21 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>GERAK</t>
+          <t>TENGAH</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Perpindahan posisi, seperti lempeng yang berpindah sangat lambat.</t>
+          <t>Batas divergen di dasar samudra disebut punggung ... samudra.</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Perpindahan tempat, seperti lempeng yang berpindah beberapa sentimeter per tahun.</t>
+          <t>Batas divergen di dasar laut disebut punggung ... laut.</t>
         </is>
       </c>
     </row>
@@ -2564,189 +2564,189 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>BENUA</t>
+          <t>LAVA</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Daratan luas, yang dahulu menyatu lalu saling menjauh.</t>
+          <t>Magma yang sudah mencapai permukaan bumi disebut...</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Daratan sangat luas yang dahulu bersatu lalu berpisah.</t>
+          <t>Zat cair panas dari dalam bumi yang sudah keluar ke permukaan.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Batas Konvergen &amp; Subduksi</t>
+          <t>Batas Divergen</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>PALUNG</t>
+          <t>MELEBAR</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Jurang sempit yang sangat dalam di dasar samudra akibat penunjaman lempeng.</t>
+          <t>Bertambah luas, seperti dasar samudra yang terus memanjang.</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Jurang sangat dalam di dasar laut, terbentuk saat lempeng menunjam.</t>
+          <t>Bertambah lebar, seperti dasar laut yang terus memanjang.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Batas Konvergen &amp; Subduksi</t>
+          <t>Batas Divergen</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>MERAPI</t>
+          <t>RETAK</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Contoh gunung berapi aktif di Indonesia yang terbentuk dari jalur subduksi lempeng.</t>
+          <t>Keadaan kerak yang terbelah akibat gaya yang menariknya memisah.</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Gunung berapi aktif di Jawa Tengah yang meletus dahsyat tahun 2010.</t>
+          <t>Keadaan kerak yang terbelah-belah karena ditarik ke dua arah.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Batas Konvergen &amp; Subduksi</t>
+          <t>Batas Divergen</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>SUBDUKSI</t>
+          <t>ZONA</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Nama proses saat lempeng samudra menunjam ke bawah lempeng benua.</t>
+          <t>Sebutan untuk daerah atau kawasan yang memiliki ciri tertentu.</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Sebutan proses penunjaman lempeng laut ke bawah lempeng daratan.</t>
+          <t>Sebutan bagi kawasan yang punya ciri khas tertentu.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
+        <v>5</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Batas Divergen</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
         <v>6</v>
       </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Batas Konvergen &amp; Subduksi</t>
-        </is>
-      </c>
-      <c r="C80" t="n">
-        <v>2</v>
-      </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>TUMBUKAN</t>
+          <t>MENGAPUNG</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Batas konvergen terjadi karena dua lempeng mengalami...</t>
+          <t>Keadaan lempeng yang berada di atas lapisan mantel yang kental.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Batas konvergen terjadi karena dua lempeng saling bertabrakan.</t>
+          <t>Keadaan lempeng yang terapung di atas lapisan kental di bawahnya.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
+        <v>5</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Batas Divergen</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
         <v>6</v>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Batas Konvergen &amp; Subduksi</t>
-        </is>
-      </c>
-      <c r="C81" t="n">
-        <v>3</v>
-      </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>MENUNJAM</t>
+          <t>GERAK</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Arah gerak lempeng samudra terhadap lempeng benua pada zona subduksi.</t>
+          <t>Perpindahan posisi, seperti lempeng yang berpindah sangat lambat.</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Arah gerak lempeng laut pada zona subduksi: menyusup ke bawah lempeng daratan.</t>
+          <t>Perpindahan tempat, seperti lempeng yang berpindah beberapa sentimeter per tahun.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
+        <v>5</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Batas Divergen</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
         <v>6</v>
       </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Batas Konvergen &amp; Subduksi</t>
-        </is>
-      </c>
-      <c r="C82" t="n">
-        <v>3</v>
-      </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>LEMPENG</t>
+          <t>BENUA</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Pecahan besar kerak bumi yang bergerak dan bertumbukan di batas konvergen.</t>
+          <t>Daratan luas, yang dahulu menyatu lalu saling menjauh.</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Potongan raksasa kerak bumi yang saling bertabrakan di batas konvergen.</t>
+          <t>Daratan sangat luas yang dahulu bersatu lalu berpisah.</t>
         </is>
       </c>
     </row>
@@ -2760,21 +2760,21 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>HIMALAYA</t>
+          <t>PALUNG</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pegunungan lipatan tertinggi di dunia, hasil tumbukan dua lempeng BENUA.</t>
+          <t>Jurang sempit yang sangat dalam di dasar samudra akibat penunjaman lempeng.</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Rangkaian pegunungan tertinggi di dunia, hasil tumbukan dua lempeng daratan.</t>
+          <t>Jurang sangat dalam di dasar laut, terbentuk saat lempeng menunjam.</t>
         </is>
       </c>
     </row>
@@ -2788,21 +2788,21 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>LIPATAN</t>
+          <t>MERAPI</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Bentuk pegunungan dari tumbukan dua lempeng benua, bukan gunung api.</t>
+          <t>Contoh gunung berapi aktif di Indonesia yang terbentuk dari jalur subduksi lempeng.</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Jenis pegunungan yang terbentuk dari tumbukan dua lempeng daratan.</t>
+          <t>Gunung berapi aktif di Jawa Tengah yang meletus dahsyat tahun 2010.</t>
         </is>
       </c>
     </row>
@@ -2816,21 +2816,21 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>TEKUK</t>
+          <t>SUBDUKSI</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Keadaan lempeng yang terlipat ke bawah saat dua lempeng bertumbukan.</t>
+          <t>Nama proses saat lempeng samudra menunjam ke bawah lempeng benua.</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Yang terjadi pada salah satu lempeng: terlipat dan masuk ke bawah lempeng lain.</t>
+          <t>Sebutan proses penunjaman lempeng laut ke bawah lempeng daratan.</t>
         </is>
       </c>
     </row>
@@ -2844,21 +2844,21 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>DAHSYAT</t>
+          <t>TUMBUKAN</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Sifat gerakan tumbukan lempeng yang menimbulkan gempa sangat kuat.</t>
+          <t>Batas konvergen terjadi karena dua lempeng mengalami...</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Sifat gerakan tumbukan lempeng hingga memicu gempa dan tsunami Aceh 2004.</t>
+          <t>Batas konvergen terjadi karena dua lempeng saling bertabrakan.</t>
         </is>
       </c>
     </row>
@@ -2872,21 +2872,21 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>GUNUNG</t>
+          <t>MENUNJAM</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Bentuk permukaan bumi yang menjulang tinggi dan sering berbentuk kerucut.</t>
+          <t>Arah gerak lempeng samudra terhadap lempeng benua pada zona subduksi.</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Bentang alam menjulang yang sering berbentuk kerucut dan dapat meletus.</t>
+          <t>Arah gerak lempeng laut pada zona subduksi: menyusup ke bawah lempeng daratan.</t>
         </is>
       </c>
     </row>
@@ -2900,21 +2900,21 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>PEGUNUNGAN</t>
+          <t>LEMPENG</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Rangkaian gunung berderet memanjang, seperti hasil tumbukan lempeng.</t>
+          <t>Pecahan besar kerak bumi yang bergerak dan bertumbukan di batas konvergen.</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Kumpulan gunung yang berderet, terbentuk dari tumbukan lempeng.</t>
+          <t>Potongan raksasa kerak bumi yang saling bertabrakan di batas konvergen.</t>
         </is>
       </c>
     </row>
@@ -2928,21 +2928,21 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>INDONESIA</t>
+          <t>HIMALAYA</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Negara kepulauan yang terbentuk dari jalur subduksi lempeng aktif.</t>
+          <t>Pegunungan lipatan tertinggi di dunia, hasil tumbukan dua lempeng BENUA.</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Kepulauan yang lahir dari tumbukan lempeng, sehingga rawan gempa dan tsunami.</t>
+          <t>Rangkaian pegunungan tertinggi di dunia, hasil tumbukan dua lempeng daratan.</t>
         </is>
       </c>
     </row>
@@ -2956,148 +2956,148 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>GEMPA</t>
+          <t>LIPATAN</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Getaran yang ditimbulkan oleh tumbukan dua lempeng kulit bumi.</t>
+          <t>Bentuk pegunungan dari tumbukan dua lempeng benua, bukan gunung api.</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Getaran kuat akibat lempeng yang saling bertumbukan, dapat memicu tsunami.</t>
+          <t>Jenis pegunungan yang terbentuk dari tumbukan dua lempeng daratan.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Batas Transform</t>
+          <t>Batas Konvergen &amp; Subduksi</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>TRANSFORM</t>
+          <t>TABRAKAN</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Batas lempeng tektonik di mana dua lempeng saling bergesekan mendatar berlawanan arah.</t>
+          <t>Batas konvergen terjadi karena ... antara dua lempeng tektonik.</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Jenis batas lempeng tempat dua lempeng saling bergesekan mendatar berlawanan arah.</t>
+          <t>Peristiwa benturan antara dua lempeng yang membentuk batas konvergen.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Batas Transform</t>
+          <t>Batas Konvergen &amp; Subduksi</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>KALIFORNIA</t>
+          <t>TINGGI</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Wilayah di Amerika Serikat tempat patahan San Andreas membentang.</t>
+          <t>Tumbukan dua lempeng benua mengangkat daratan menjadi pegunungan yang sangat...</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Nama wilayah tempat sesar San Andreas berada.</t>
+          <t>Akibat benturan dua lempeng daratan, tanah terangkat sampai menjulang ke langit.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Batas Transform</t>
+          <t>Batas Konvergen &amp; Subduksi</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>INCI</t>
+          <t>GUNUNG</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Satuan panjang; sesar San Andreas bergeser sekitar 2 ... per tahun.</t>
+          <t>Bentuk permukaan bumi yang menjulang tinggi dan sering berbentuk kerucut.</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Satuan panjang pergeseran San Andreas setiap tahun (2 ... per tahun).</t>
+          <t>Bentang alam menjulang yang sering berbentuk kerucut dan dapat meletus.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Batas Transform</t>
+          <t>Batas Konvergen &amp; Subduksi</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>SESAR</t>
+          <t>PEGUNUNGAN</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Nama lain patahan mendatar tempat dua lempeng bergesekan menyamping.</t>
+          <t>Rangkaian gunung berderet memanjang, seperti hasil tumbukan lempeng.</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Sebutan lain bagi patahan mendatar, tempat dua lempeng bergesekan menyamping.</t>
+          <t>Kumpulan gunung yang berderet, terbentuk dari tumbukan lempeng.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
+        <v>6</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Batas Konvergen &amp; Subduksi</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
         <v>7</v>
       </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Batas Transform</t>
-        </is>
-      </c>
-      <c r="C95" t="n">
-        <v>3</v>
-      </c>
       <c r="D95" t="inlineStr">
         <is>
           <t>DANGKAL</t>
@@ -3105,40 +3105,40 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Sifat gempa yang dipicu oleh gesekan di batas transform.</t>
+          <t>Sifat gempa yang pusatnya dekat permukaan, sehingga getarannya kuat.</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Sifat gempa akibat gesekan batuan yang terlepas di batas transform.</t>
+          <t>Sifat gempa yang pusatnya dekat permukaan bumi; getarannya terasa kuat.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
+        <v>6</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Batas Konvergen &amp; Subduksi</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
         <v>7</v>
       </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Batas Transform</t>
-        </is>
-      </c>
-      <c r="C96" t="n">
-        <v>3</v>
-      </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>ENERGI</t>
+          <t>MENDEKAT</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Yang dilepaskan ketika gesekan batuan di sesar tidak lagi tertahan.</t>
+          <t>Arah gerak dua lempeng pada batas konvergen, yaitu saling...</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Yang terlepas saat batuan di sepanjang sesar bergesekan lalu retak.</t>
+          <t>Pada batas konvergen, kedua lempeng bergerak saling menghampiri.</t>
         </is>
       </c>
     </row>
@@ -3152,21 +3152,21 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>BERGESEK</t>
+          <t>TRANSFORM</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Dua lempeng pada batas transform saling ... mendatar.</t>
+          <t>Batas lempeng tektonik di mana dua lempeng saling bergesekan mendatar berlawanan arah.</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Kedua lempeng bersentuhan dan saling menggosok menyamping di batas transform.</t>
+          <t>Jenis batas lempeng tempat dua lempeng saling bergesekan mendatar berlawanan arah.</t>
         </is>
       </c>
     </row>
@@ -3180,21 +3180,21 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>BATUAN</t>
+          <t>SANANDREAS</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Bahan yang saling bergesekan di sepanjang sesar pada batas transform.</t>
+          <t>Patahan mendatar terkenal di California yang membentang sepanjang 1.200 kilometer.</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Yang saling bergesekan di sepanjang sesar sehingga memicu gempa.</t>
+          <t>Patahan mendatar di California yang panjangnya sekitar 1.200 kilometer.</t>
         </is>
       </c>
     </row>
@@ -3208,21 +3208,21 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>LEPAS</t>
+          <t>GESERAN</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Nasib energi gesekan batuan ketika sudah tidak tertahan lagi.</t>
+          <t>Jenis pergerakan lempeng pada batas transform: ... mendatar.</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Energi gesekan batuan akan ... dan memicu gempa dangkal.</t>
+          <t>Pada batas transform, lempeng bergerak menyamping sejajar permukaan bumi.</t>
         </is>
       </c>
     </row>
@@ -3236,21 +3236,21 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>SEJAJAR</t>
+          <t>SESAR</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Posisi dua garis yang arahnya sama dan tidak pernah berpotongan.</t>
+          <t>Nama lain patahan mendatar tempat dua lempeng bergesekan menyamping.</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Kedudukan dua garis yang arahnya sama dan tak pernah bertemu.</t>
+          <t>Sebutan lain bagi patahan mendatar, tempat dua lempeng bergesekan menyamping.</t>
         </is>
       </c>
     </row>
@@ -3264,21 +3264,21 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>DATAR</t>
+          <t>MENDATAR</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Kedudukan kedua lempeng pada batas transform: sejajar dan rata.</t>
+          <t>Arah gesekan kedua lempeng pada batas transform: saling bergesekan...</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Posisi kedua lempeng yang bergesek di batas transform: sama ...</t>
+          <t>Arah gesekan kedua lempeng pada batas transform, yaitu sejajar permukaan.</t>
         </is>
       </c>
     </row>
@@ -3292,21 +3292,189 @@
         </is>
       </c>
       <c r="C102" t="n">
+        <v>3</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>PATAHAN</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Retakan panjang di kerak bumi akibat gesekan mendatar lempeng.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Retakan panjang di kerak akibat dua lempeng bergesekan menyamping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>7</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Batas Transform</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>4</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>BERGESEK</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Dua lempeng pada batas transform saling ... mendatar.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Kedua lempeng bersentuhan dan saling menggosok menyamping di batas transform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>7</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Batas Transform</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>4</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>PATAH</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Batuan di sepanjang sesar dapat ... dan melepaskan energi gempa.</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Ketika batuan di sepanjang sesar tak kuat lagi menahan, energi gempa terlepas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>7</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Batas Transform</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>5</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>HORIZONTAL</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Arah gesekan kedua lempeng pada batas transform, yaitu mendatar.</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Arah gesekan kedua lempeng pada batas transform: sejajar permukaan bumi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>7</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Batas Transform</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>5</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>SEJAJAR</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Posisi dua garis yang arahnya sama dan tidak pernah berpotongan.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Kedudukan dua garis yang arahnya sama dan tak pernah bertemu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>7</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Batas Transform</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
         <v>6</v>
       </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>POSISI</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Letak kedua lempeng ketika bergesekan: dalam ... yang sama.</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>Kedudukan kedua lempeng saat bergesek: dalam ... yang sama rata.</t>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>REKAH</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Keadaan tanah yang terbelah-belah akibat gesekan lempeng mendatar.</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Keadaan tanah yang pecah-pecah akibat gesekan lempeng mendatar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>7</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Batas Transform</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>6</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>TEGANGAN</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Yang menumpuk pada batuan akibat gesekan yang terus-menerus.</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Yang terkumpul pada batuan karena gesekan terus-menerus, lalu dilepas saat retak.</t>
         </is>
       </c>
     </row>
@@ -3393,22 +3561,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MERUNDUK</t>
+          <t>BERLINDUNG</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Gerakan pertama saat gempa: ... ke bawah mendekati lantai agar tidak terkena benda yang jatuh.</t>
+          <t>Masuk ke bawah meja saat terjadi gempa untuk ... dari material yang jatuh.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Gerakan menurunkan badan mendekati lantai saat gempa dimulai.</t>
+          <t>Tindakan mencari tempat aman di bawah meja agar tidak tertimpa benda yang jatuh.</t>
         </is>
       </c>
     </row>
@@ -3434,17 +3602,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>KORSLETING</t>
+          <t>EVAKUASI</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Bahaya listrik yang harus diwaspadai setelah guncangan mereda.</t>
+          <t>Penyelamatan diri dengan berjalan tertib lewat tangga darurat menuju titik kumpul di lapangan sekolah.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Risiko hubungan arus pendek yang diperiksa sebelum meninggalkan area.</t>
+          <t>Upaya menyelamatkan diri menuju titik kumpul dengan tertib lewat jalur darurat.</t>
         </is>
       </c>
     </row>
@@ -3465,22 +3633,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>BERLINDUNG</t>
+          <t>GEMPA</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Masuk ke bawah meja saat terjadi gempa untuk ... dari material yang jatuh.</t>
+          <t>Peristiwa getaran atau guncangan tanah mendadak yang kita simulasikan cara penyelamatannya di kelas.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Tindakan mencari tempat aman di bawah meja agar tidak tertimpa benda yang jatuh.</t>
+          <t>Guncangan tanah yang datang mendadak dan dapat merobohkan bangunan.</t>
         </is>
       </c>
     </row>
@@ -3501,22 +3669,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>EVAKUASI</t>
+          <t>SIAGA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Saat status AWAS, segera tinggalkan zona KRB III menuju tempat aman.</t>
+          <t>Tas darurat 72 jam yang diajarkan Bu Rahma berisi makanan, air, dan obat disebut Tas ... Bencana.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Tindakan meninggalkan kawasan berbahaya ke tempat aman ketika status AWAS.</t>
+          <t>Tas berisi makanan, air, dan obat untuk 72 jam pertama, disebut Tas ... Bencana.</t>
         </is>
       </c>
     </row>
@@ -3537,22 +3705,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PELUIT</t>
+          <t>MERUNDUK</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Alat yang dibunyikan untuk meminta pertolongan saat terjebak.</t>
+          <t>Gerakan pertama saat gempa: ... ke bawah mendekati lantai agar tidak terkena benda yang jatuh.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Benda kecil di tas siaga yang bunyinya memanggil bantuan.</t>
+          <t>Gerakan menurunkan badan mendekati lantai saat gempa dimulai.</t>
         </is>
       </c>
     </row>
@@ -3573,22 +3741,22 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SENTER</t>
+          <t>RINGAN</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alat penerang di dalam tas siaga bencana.</t>
+          <t>Sebutan untuk gempa berkekuatan kecil, yang getarannya hanya dirasakan sebagian orang.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Perkakas bercahaya yang wajib ada di tas siaga untuk keadaan gelap.</t>
+          <t>Sebutan gempa berkekuatan kecil; getarannya hanya terasa oleh sebagian orang.</t>
         </is>
       </c>
     </row>
@@ -3609,22 +3777,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TANGGA</t>
+          <t>RENCANA</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Jalur turun darurat yang dipakai saat gempa, dan bukan lift.</t>
+          <t>Susunan langkah yang disiapkan jauh sebelum bencana terjadi, misalnya ... evakuasi sekolah.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Jalur menurun di gedung yang wajib dipakai saat evakuasi, bukan lift.</t>
+          <t>Sebelum bencana datang, sekolah menyusun ini agar tahu apa yang harus dilakukan: ... evakuasi.</t>
         </is>
       </c>
     </row>
@@ -3650,17 +3818,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>RANSUM</t>
+          <t>UPAYA</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Makanan darurat yang disimpan di dalam tas siaga bencana.</t>
+          <t>Ikhtiar yang dilakukan manusia untuk mengurangi risiko bencana, misalnya latihan evakuasi rutin.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Bekal makanan tahan lama untuk 72 jam pertama.</t>
+          <t>Ikhtiar manusia untuk menekan risiko bencana, contohnya latihan berkala.</t>
         </is>
       </c>
     </row>
@@ -3686,17 +3854,17 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>GEMPA</t>
+          <t>BANGUNAN</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Peristiwa getaran atau guncangan tanah mendadak yang kita simulasikan cara penyelamatannya di kelas.</t>
+          <t>Struktur yang wajib dirancang tahan gempa di daerah rawan gempa.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Guncangan tanah yang datang mendadak dan dapat merobohkan bangunan.</t>
+          <t>Struktur buatan manusia yang wajib dirancang tahan guncangan di daerah rawan.</t>
         </is>
       </c>
     </row>
@@ -3722,17 +3890,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SIAGA</t>
+          <t>LATIHAN</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Tingkat status gunung api Level III yang menunjukkan peningkatan aktivitas seismik secara nyata dan letusan dapat segera menyusul.</t>
+          <t>Kegiatan mengulang prosedur evakuasi agar menjadi kebiasaan saat panik.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Tingkat status gunung api Level III: aktivitas gempa meningkat nyata, letusan dapat menyusul.</t>
+          <t>Kegiatan mengulang prosedur penyelamatan diri agar terbiasa saat panik.</t>
         </is>
       </c>
     </row>
@@ -3758,17 +3926,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TERTIB</t>
+          <t>PERSIAPAN</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Sikap berbaris rapi tanpa saling mendorong ketika evakuasi.</t>
+          <t>Segala usaha yang dilakukan SEBELUM bencana terjadi agar risiko berkurang.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Cara berjalan menuju titik kumpul: rapi dan tidak saling dorong.</t>
+          <t>Semua yang dikerjakan jauh hari sebelum bencana, supaya risikonya mengecil.</t>
         </is>
       </c>
     </row>
@@ -3789,22 +3957,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>DENAH</t>
+          <t>PETUGAS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Gambar susunan ruangan yang dipelajari agar tahu jalur keluar.</t>
+          <t>Orang yang bertugas menertibkan warga saat evakuasi berlangsung.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Yang dikenali sejak sebelum gempa supaya tahu jalan keluar sekolah.</t>
+          <t>Orang yang bertugas menertibkan warga saat proses penyelamatan berlangsung.</t>
         </is>
       </c>
     </row>
@@ -4257,22 +4425,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SELAMAT</t>
+          <t>SUSULAN</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Kondisi warga yang berhasil keluar dari bangunan tanpa cedera.</t>
+          <t>Getaran gempa bumi berikutnya yang berpotensi terjadi beberapa menit hingga beberapa hari setelah gempa utama.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Keadaan warga yang berhasil keluar dari bangunan tanpa luka sedikit pun.</t>
+          <t>Getaran lanjutan setelah gempa utama, dapat terjadi beberapa menit sampai beberapa hari.</t>
         </is>
       </c>
     </row>
@@ -4298,17 +4466,17 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SUSULAN</t>
+          <t>LAPANGAN</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Getaran gempa bumi berikutnya yang berpotensi terjadi beberapa menit hingga beberapa hari setelah gempa utama.</t>
+          <t>Area terbuka luas yang paling aman dijadikan titik kumpul warga sekolah karena terbebas dari bahaya reruntuhan bangunan.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Getaran lanjutan setelah gempa utama, dapat terjadi beberapa menit sampai beberapa hari.</t>
+          <t>Area terbuka luas yang paling aman sebagai titik kumpul karena bebas reruntuhan.</t>
         </is>
       </c>
     </row>
@@ -4329,22 +4497,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>PRESENSI</t>
+          <t>BMKG</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Pemeriksaan menyeluruh di titik kumpul untuk memastikan tidak ada yang tertinggal.</t>
+          <t>Lembaga resmi pemerintah yang berwenang menyiarkan informasi gempa bumi dan peringatan dini tsunami di Indonesia.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Pendataan ulang seluruh siswa di titik kumpul agar tidak ada yang hilang.</t>
+          <t>Lembaga pemerintah yang menyiarkan informasi gempa dan peringatan dini tsunami.</t>
         </is>
       </c>
     </row>
@@ -4365,22 +4533,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>KOORDINATOR</t>
+          <t>MEDIS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Orang yang memimpin pemeriksaan di titik kumpul.</t>
+          <t>Bantuan pertolongan pertama (P3K) dan perawatan kesehatan yang diberikan kepada korban luka atau syok di posko darurat.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Pihak yang mengatur pendataan warga di titik kumpul bersama guru.</t>
+          <t>Bantuan pertolongan pertama dan perawatan kesehatan bagi korban luka di posko.</t>
         </is>
       </c>
     </row>
@@ -4406,17 +4574,17 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>HOAKS</t>
+          <t>KEHADIRAN</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Kabar bohong yang harus dihindari dan tidak disebarkan.</t>
+          <t>Hal pertama yang diperiksa di titik kumpul, apakah semua sudah lengkap.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Informasi palsu yang wajib tidak diteruskan ke orang lain.</t>
+          <t>Di titik kumpul, petugas menghitung orang untuk memastikan tidak ada yang tertinggal.</t>
         </is>
       </c>
     </row>
@@ -4437,22 +4605,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>KORBAN</t>
+          <t>BERKUMPUL</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Orang yang mengalami luka atau kerugian akibat peristiwa bencana.</t>
+          <t>Setelah guncangan usai, semua warga menuju lapangan agar mudah diperiksa.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Siapa pun yang terkena dampak bencana, baik terluka maupun kehilangan harta.</t>
+          <t>Petugas memeriksa kelengkapan warga tepat setelah guncangan reda, di tempat terbuka.</t>
         </is>
       </c>
     </row>
@@ -4473,22 +4641,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>RETAK</t>
+          <t>RERUNTUHAN</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Keadaan bangunan yang harus dijauhi setelah gempa.</t>
+          <t>Puing bangunan yang menutup jalur evakuasi setelah gempa besar.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Kondisi dinding gedung yang menandakan strukturnya belum aman.</t>
+          <t>Sisa bangunan yang runtuh dan menghalangi jalan keluar.</t>
         </is>
       </c>
     </row>
@@ -4509,22 +4677,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>MEDIS</t>
+          <t>AMBULANS</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Bantuan pertolongan pertama (P3K) dan perawatan kesehatan yang diberikan kepada korban luka atau syok di posko darurat.</t>
+          <t>Kendaraan pengangkut korban luka menuju rumah sakit terdekat.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Bantuan pertolongan pertama dan perawatan kesehatan bagi korban luka di posko.</t>
+          <t>Kendaraan bersirine yang membawa orang terluka ke rumah sakit.</t>
         </is>
       </c>
     </row>
@@ -4545,22 +4713,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>KABEL</t>
+          <t>KORBAN</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Yang harus dijauhi bersama tiang dan pohon agar tidak tersengat.</t>
+          <t>Orang yang mengalami luka atau kerugian akibat peristiwa bencana.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Saluran listrik yang berbahaya bila tersentuh setelah gempa.</t>
+          <t>Siapa pun yang terkena dampak bencana, baik terluka maupun kehilangan harta.</t>
         </is>
       </c>
     </row>
@@ -4586,17 +4754,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>BMKG</t>
+          <t>POSKO</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Lembaga resmi pemerintah yang berwenang menyiarkan informasi gempa bumi dan peringatan dini tsunami di Indonesia.</t>
+          <t>Tempat penanganan darurat yang didirikan di lapangan evakuasi.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Lembaga pemerintah yang menyiarkan informasi gempa dan peringatan dini tsunami.</t>
+          <t>Tempat penanganan darurat yang didirikan di area titik kumpul.</t>
         </is>
       </c>
     </row>
@@ -4622,17 +4790,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>LUKA</t>
+          <t>PETUGAS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Keadaan korban yang mendapat pertolongan pertama setelah gempa.</t>
+          <t>Orang berkompeten yang dipanggil untuk menangani korban cedera.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Akibat yang dialami korban sehingga perlu bantuan medis.</t>
+          <t>Pihak yang dipanggil karena keahliannya untuk merawat orang terluka.</t>
         </is>
       </c>
     </row>
@@ -4658,17 +4826,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>GURU</t>
+          <t>SELAMAT</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Yang melakukan presensi bersama koordinator di titik kumpul.</t>
+          <t>Kondisi warga yang berhasil keluar dari bangunan tanpa cedera.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Pendamping siswa yang memastikan semua anak terdata di titik kumpul.</t>
+          <t>Keadaan warga yang berhasil keluar dari bangunan tanpa luka sedikit pun.</t>
         </is>
       </c>
     </row>
@@ -4689,22 +4857,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>MASKER</t>
+          <t>MAGMA</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Alat yang menutup hidung dan mulut untuk menyaring abu vulkanik.</t>
+          <t>Batuan cair pijar bersuhu ribuan derajat di perut bumi, sekaligus nama aplikasi resmi pemantauan gunung api di Indonesia.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Pelindung pernapasan yang wajib dikenakan saat status SIAGA.</t>
+          <t>Zat cair pijar bersuhu ribuan derajat di perut bumi, juga nama aplikasi pemantauan gunung api.</t>
         </is>
       </c>
     </row>
@@ -4725,22 +4893,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>WASPADA</t>
+          <t>MASKER</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Tingkat status gunung api satu langkah di atas Normal.</t>
+          <t>Alat pelindung pernapasan wajib disiapkan untuk menyaring partikel abu silika tajam agar tidak merusak paru-paru.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Tingkat status gunung api satu tingkat di atas Normal, yaitu Level II.</t>
+          <t>Alat pelindung pernapasan untuk menyaring abu tajam agar paru-paru tidak rusak.</t>
         </is>
       </c>
     </row>
@@ -4766,17 +4934,17 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>AWAS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Tingkat kondisi gunung api, dari Normal sampai Awas.</t>
+          <t>Tingkat status aktivitas gunung api tertinggi (Level IV) yang menandakan letusan utama berpeluang besar segera terjadi.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Tingkat kondisi gunung api, mulai dari Normal hingga Awas.</t>
+          <t>Tingkat status gunung api tertinggi, Level IV, tanda letusan utama segera terjadi.</t>
         </is>
       </c>
     </row>
@@ -4797,22 +4965,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PANTAU</t>
+          <t>SIAGA</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Kegiatan mengamati gunung api terus-menerus dari pos pengamatan.</t>
+          <t>Tingkat status gunung api Level III yang menunjukkan peningkatan aktivitas seismik secara nyata dan letusan dapat segera menyusul.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Kegiatan mengawasi gunung api tanpa henti dari pos pengamatan.</t>
+          <t>Tingkat status gunung api Level III: aktivitas gempa meningkat nyata, letusan dapat menyusul.</t>
         </is>
       </c>
     </row>
@@ -4838,17 +5006,17 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>HUNIAN</t>
+          <t>DEFORMASI</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>KRB III adalah zona larangan ... tetap karena selalu terancam awan panas.</t>
+          <t>Perubahan bentuk tubuh gunung akibat tekanan magma dari dalam.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Jenis bangunan yang dilarang berdiri tetap di KRB III.</t>
+          <t>Perubahan bentuk tubuh gunung akibat tekanan zat cair panas dari dalam.</t>
         </is>
       </c>
     </row>
@@ -4874,17 +5042,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>GEMBEL</t>
+          <t>WASPADA</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Kata kedua dari sebutan Jawa untuk awan panas: wedhus ...</t>
+          <t>Tingkat status gunung api satu langkah di atas Normal.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Pasangan kata "wedhus", nama lain awan panas guguran.</t>
+          <t>Tingkat status gunung api satu tingkat di atas Normal, yaitu Level II.</t>
         </is>
       </c>
     </row>
@@ -4910,17 +5078,17 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>LERENG</t>
+          <t>SEISMOGRAF</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Bagian miring gunung tempat KRB II berada.</t>
+          <t>Alat perekam getaran magma di pos pengamatan gunung api.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Bagian gunung yang melandai di bawah puncak, termasuk zona tengah.</t>
+          <t>Di pos pengamatan, alat ini mencatat setiap getaran yang berasal dari dalam gunung.</t>
         </is>
       </c>
     </row>
@@ -4946,17 +5114,17 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>GOGGLE</t>
+          <t>STATUS</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Kacamata pelindung yang wajib dipakai bersama masker N95.</t>
+          <t>Tingkat kondisi gunung api, dari Normal sampai Awas.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Pelindung mata dari abu vulkanik, bagian dari APD warga Merapi.</t>
+          <t>Tingkat kondisi gunung api, mulai dari Normal hingga Awas.</t>
         </is>
       </c>
     </row>
@@ -4982,17 +5150,17 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>PVMBG</t>
+          <t>KABUT</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Lembaga pemerintah yang memantau aktivitas gunung api di Indonesia.</t>
+          <t>Sebutan sehari-hari untuk awan panas yang meluncur dari kawah.</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Nama lembaga yang berwenang mengeluarkan status gunung api di negara kita.</t>
+          <t>Warga biasa menyebut awan panas yang turun dari kawah dengan kata ini.</t>
         </is>
       </c>
     </row>
@@ -5018,17 +5186,17 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>SIAGA</t>
+          <t>GAS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Tingkat status gunung api Level III yang menunjukkan peningkatan aktivitas seismik secara nyata dan letusan dapat segera menyusul.</t>
+          <t>Zat yang komposisinya dipantau untuk menilai kesiapan gunung meletus.</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Tingkat status gunung api Level III: aktivitas gempa meningkat nyata, letusan dapat menyusul.</t>
+          <t>Zat yang keluar dari kawah dan komposisinya dipantau untuk menilai kesiapan letusan.</t>
         </is>
       </c>
     </row>
@@ -5054,17 +5222,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>MAGMA</t>
+          <t>PANTAU</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Batuan cair pijar bersuhu ribuan derajat di perut bumi, sekaligus nama aplikasi resmi pemantauan gunung api di Indonesia.</t>
+          <t>Kegiatan mengamati gunung api terus-menerus dari pos pengamatan.</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Zat cair pijar bersuhu ribuan derajat di perut bumi, juga nama aplikasi pemantauan gunung api.</t>
+          <t>Kegiatan mengawasi gunung api tanpa henti dari pos pengamatan.</t>
         </is>
       </c>
     </row>
@@ -5090,17 +5258,17 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AWAS</t>
+          <t>PVMBG</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Tingkat status aktivitas gunung api tertinggi (Level IV) yang menandakan letusan utama berpeluang besar segera terjadi.</t>
+          <t>Lembaga pemerintah yang memantau aktivitas gunung api di Indonesia.</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Tingkat status gunung api tertinggi, Level IV, tanda letusan utama segera terjadi.</t>
+          <t>Nama lembaga yang berwenang mengeluarkan status gunung api di negara kita.</t>
         </is>
       </c>
     </row>
@@ -5126,17 +5294,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>MUNTAHAN</t>
+          <t>MENGUNGSI</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Material yang disemburkan gunung ke luar saat erupsi memuncak.</t>
+          <t>Meninggalkan rumah menuju tempat aman atas arahan petugas.</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Yang keluar dari kawah ketika letusan mencapai puncaknya.</t>
+          <t>Apa yang dilakukan warga ketika petugas meminta mereka pergi ke tempat yang lebih aman.</t>
         </is>
       </c>
     </row>
@@ -5162,17 +5330,17 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>KENDARAAN</t>
+          <t>PIROKLASTIK</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Alat angkut yang dipakai warga untuk keluar dari zona KRB III.</t>
+          <t>Aliran gas dan material panas yang meluncur cepat menuruni lereng gunung.</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Saat status AWAS, warga meninggalkan zona KRB III menggunakan ...</t>
+          <t>Campuran awan gas dan batuan panas yang melesat turun dari puncak.</t>
         </is>
       </c>
     </row>
@@ -5198,17 +5366,17 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>KACAMATA</t>
+          <t>PERINGATAN</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Pelindung mata dari abu vulkanik, dipakai bersama masker.</t>
+          <t>Pemberitahuan resmi mengenai ancaman bahaya yang akan datang.</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Alat yang menutup kedua mata agar abu vulkanik tidak melukai kornea.</t>
+          <t>Kabar resmi dari pihak berwenang bahwa bahaya sedang mendekat.</t>
         </is>
       </c>
     </row>
@@ -5234,17 +5402,17 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>EVAKUASI</t>
+          <t>LEDAKAN</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Saat status AWAS, segera tinggalkan zona KRB III menuju tempat aman.</t>
+          <t>Letusan dahsyat yang menyemburkan material vulkanik ke udara.</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Tindakan meninggalkan kawasan berbahaya ke tempat aman ketika status AWAS.</t>
+          <t>Peristiwa letusan hebat yang menyemburkan material vulkanik ke udara.</t>
         </is>
       </c>
     </row>
@@ -5270,17 +5438,17 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>MASKER</t>
+          <t>GEMURUH</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Alat yang menutup hidung dan mulut untuk menyaring abu vulkanik.</t>
+          <t>Suara berdengung keras dari dalam gunung tanda aktivitas meningkat.</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Pelindung pernapasan yang wajib dikenakan saat status SIAGA.</t>
+          <t>Bunyi berat dari perut gunung yang menandakan aktivitasnya naik.</t>
         </is>
       </c>
     </row>
@@ -5306,17 +5474,17 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>TREMOR</t>
+          <t>ERUPSI</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Getaran halus dari dalam gunung yang mendahului erupsi.</t>
+          <t>Peristiwa keluarnya magma dan gas dari dalam gunung menuju permukaan.</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Gempa kecil terus-menerus yang menjadi tanda awal gunung akan meletus.</t>
+          <t>Peristiwa keluarnya zat cair panas dan gas dari gunung ke permukaan.</t>
         </is>
       </c>
     </row>
@@ -5337,22 +5505,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>TUTUP</t>
+          <t>MENURUN</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Tindakan pada jendela dan pintu agar abu tidak masuk ke rumah.</t>
+          <t>Arah aliran awan panas, yaitu mengikuti lereng dan lembah.</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Yang dilakukan pada jendela agar abu vulkanik tidak masuk.</t>
+          <t>Arah aliran awan panas: bergerak turun mengikuti lereng dan lembah.</t>
         </is>
       </c>
     </row>
@@ -5378,17 +5546,17 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>ERUPSI</t>
+          <t>KRATER</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Peristiwa keluarnya magma dan gas dari gunung ke permukaan.</t>
+          <t>Lubang kawah di puncak gunung tempat magma dan gas keluar.</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Peristiwa letusan gunung api yang mengeluarkan magma dan abu.</t>
+          <t>Lubang kawah di puncak gunung tempat zat cair panas dan gas keluar.</t>
         </is>
       </c>
     </row>
@@ -5414,17 +5582,17 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>PANIK</t>
+          <t>LAHAR</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Kondisi gelisah hewan liar yang menjadi tanda awal erupsi.</t>
+          <t>Aliran campuran air, pasir, dan batu vulkanik yang turun melalui alur sungai.</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Keadaan berlarian binatang di lereng gunung sebelum letusan.</t>
+          <t>Ketika hujan bercampur material vulkanik mengalir deras menyusuri lembah sungai.</t>
         </is>
       </c>
     </row>
@@ -5445,22 +5613,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>SATWA</t>
+          <t>TUTUP</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Hewan liar di lereng gunung yang gelisah dan turun ke desa sebelum letusan.</t>
+          <t>Yang harus dilakukan pada jendela dan pintu agar abu tidak masuk.</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Binatang yang panik dan turun gunung menjelang erupsi.</t>
+          <t>Tindakan pada jendela dan pintu agar abu tidak masuk ke rumah.</t>
         </is>
       </c>
     </row>
@@ -5481,22 +5649,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>ASAP</t>
+          <t>SUMBER</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Tanda awal erupsi: keluar ... putih dari puncak gunung.</t>
+          <t>Tempat air berasal, yang wajib dilindungi dari abu vulkanik.</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Yang mengepul dari kawah; putih saat WASPADA, kelabu pekat saat SIAGA.</t>
+          <t>Tempat air berasal dan wajib dilindungi agar tidak tercemar abu.</t>
         </is>
       </c>
     </row>
@@ -5517,22 +5685,22 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>LAYU</t>
+          <t>BAHAYA</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Keadaan tumbuhan akibat panas tanah sebelum gunung meletus.</t>
+          <t>Kondisi yang mengancam keselamatan sehingga warga harus menjauh.</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Yang terjadi pada tanaman karena tanah menjadi panas menjelang letusan.</t>
+          <t>Keadaan yang mengancam keselamatan sehingga warga wajib menjauh.</t>
         </is>
       </c>
     </row>
@@ -5553,22 +5721,22 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>TANDON</t>
+          <t>BARAK</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Wadah besar penampung air bersih yang harus dijaga kebersihannya.</t>
+          <t>Tempat penampungan pengungsian terpadu yang aman bagi warga terdampak erupsi, dilengkapi posko medis dan logistik.</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Tempat penampungan air bersih yang harus dijaga kebersihannya.</t>
+          <t>Tempat penampungan terpadu yang aman bagi warga terdampak letusan, lengkap dengan posko.</t>
         </is>
       </c>
     </row>
@@ -5589,22 +5757,22 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>PENGUNGSI</t>
+          <t>ATAP</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Warga yang meninggalkan rumah dan tinggal sementara di tempat penampungan.</t>
+          <t>Bagian bangunan rumah yang wajib dibersihkan dari timbunan abu vulkanik tebal secara gotong royong agar tidak ambruk akibat beban berat.</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Warga yang untuk sementara tidak tinggal di rumahnya karena mencari tempat aman.</t>
+          <t>Bagian teratas rumah yang wajib dibersihkan dari timbunan abu agar tidak ambruk.</t>
         </is>
       </c>
     </row>
@@ -5625,22 +5793,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>GOTONG</t>
+          <t>PAPAN</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Sikap bersama-sama warga saat membersihkan atap dari abu: ... royong.</t>
+          <t>Alas panjang beralas kain yang dipakai petugas mengusung korban luka ke posko medis, disebut tandu darurat.</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Cara warga membersihkan atap secara bersama-sama.</t>
+          <t>Tandu darurat: alas berkain yang dipakai petugas mengusung orang terluka ke posko.</t>
         </is>
       </c>
     </row>
@@ -5666,17 +5834,17 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>SANITASI</t>
+          <t>AMAN</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Sistem kebersihan di penampungan yang wajib dijaga agar penyakit tidak menyebar.</t>
+          <t>Keadaan warga di barak pengungsian Zona KRB I yang terbebas dari bahaya awan panas dan guguran lava.</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Di penampungan, air bersih dan pembuangan sampah harus dijaga agar wabah tidak muncul.</t>
+          <t>Warga di barak Zona KRB I jauh dari jangkauan awan panas maupun guguran lava.</t>
         </is>
       </c>
     </row>
@@ -5702,17 +5870,17 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>WEDHUS</t>
+          <t>BANTUAN</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Kata Jawa di depan "gembel", nama lain awan panas guguran.</t>
+          <t>Kiriman kebutuhan yang dibagi menurut kebutuhan, bukan siapa yang cepat.</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Sebutan Jawa untuk awan panas guguran: ... gembel.</t>
+          <t>Barang kiriman yang dibagikan sesuai keperluan tiap keluarga, bukan siapa yang paling cepat mengantre.</t>
         </is>
       </c>
     </row>
@@ -5738,17 +5906,17 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>SILIKA</t>
+          <t>LOGISTIK</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Senyawa dalam abu vulkanik yang tajam dan dapat melukai paru-paru.</t>
+          <t>Pasokan kebutuhan pokok bagi para pengungsi di barak.</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Bahan dalam abu vulkanik yang berbentuk pecahan kaca mikroskopis.</t>
+          <t>Pasokan kebutuhan pokok bagi warga yang tinggal di penampungan.</t>
         </is>
       </c>
     </row>
@@ -5769,22 +5937,22 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>menurun</t>
+          <t>mendatar</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>LEMBAH</t>
+          <t>PENGUNGSI</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Bentuk bentang alam yang dilalui awan panas guguran saat meluncur turun.</t>
+          <t>Warga yang meninggalkan rumah dan tinggal di tempat penampungan.</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Awan panas guguran meluncur deras menyusuri ... sungai.</t>
+          <t>Warga yang untuk sementara tidak tinggal di rumahnya karena harus mencari tempat aman.</t>
         </is>
       </c>
     </row>
@@ -5805,22 +5973,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>AMBRUK</t>
+          <t>SANITASI</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Risiko pada atap rumah karena beban abu yang sangat berat, terutama saat basah.</t>
+          <t>Sistem kebersihan yang wajib dijaga agar penyakit tidak menyebar.</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Yang terjadi pada atap rumah bila timbunan abu tidak dibersihkan.</t>
+          <t>Di penampungan, air bersih, jamban, dan pembuangan sampah harus dijaga agar wabah tidak muncul.</t>
         </is>
       </c>
     </row>
@@ -5846,17 +6014,17 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>PARU</t>
+          <t>MEDIS</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Organ tubuh yang rusak bila menghirup abu vulkanik tanpa pelindung.</t>
+          <t>Layanan kesehatan yang wajib tersedia di barak pengungsian.</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Bagian tubuh yang paling terancam oleh pecahan kaca mikroskopis dalam abu.</t>
+          <t>Layanan kesehatan yang wajib tersedia di tempat penampungan.</t>
         </is>
       </c>
     </row>
@@ -5877,22 +6045,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>mendatar</t>
+          <t>menurun</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>TAJAM</t>
+          <t>TRAUMA</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Sifat butiran abu vulkanik yang dapat melukai kornea mata.</t>
+          <t>Gangguan jiwa akibat bencana yang memerlukan dukungan psikologis.</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Sifat pecahan kaca mikroskopis di dalam abu vulkanik.</t>
+          <t>Luka batin yang dialami penyintas bencana dan butuh pendampingan psikolog.</t>
         </is>
       </c>
     </row>
@@ -5918,17 +6086,17 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>ATAP</t>
+          <t>TANDON</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Bagian teratas rumah yang wajib dibersihkan dari timbunan abu agar tidak ambruk.</t>
+          <t>Tempat penampungan air bersih yang harus dijaga kebersihannya.</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Bagian rumah yang paling menanggung beban timbunan abu vulkanik.</t>
+          <t>Wadah besar penampung air bersih yang harus dijaga kebersihannya.</t>
         </is>
       </c>
     </row>
@@ -5954,17 +6122,17 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>DEBU</t>
+          <t>LANSIA</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Endapan vulkanik halus yang menumpuk tebal di atap rumah.</t>
+          <t>Kelompok lanjut usia yang perlu didahulukan menerima bantuan.</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Butiran sangat halus dari letusan yang mengendap di atap dan jalan.</t>
+          <t>Kelompok warga yang sudah berumur dan perlu didahulukan menerima bantuan.</t>
         </is>
       </c>
     </row>
@@ -6002,7 +6170,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>101 kata di 8 zona (Level 1)</t>
+          <t>107 kata di 8 zona (Level 1)</t>
         </is>
       </c>
     </row>

</xml_diff>